<commit_message>
feat(exp36-41): freeze official fusion line and unify Leave-Next cohort
Publish Exp36–40 challenge fusion/CSV hardening code and materials, Exp41 real-subject Leave-Next F5 cohort tooling and reports, 45ch preprocess helpers, and Exp36 summary JSON (weights excluded).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/资料/初赛材料/02_离线验证/离线性能验证报告_XH-202610.xlsx
+++ b/资料/初赛材料/02_离线验证/离线性能验证报告_XH-202610.xlsx
@@ -18,6 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_原始数据索引" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_复现与截图" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_数据核对" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_指定集Exp34_40" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -510,21 +511,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="30.3" customWidth="1" min="3" max="3"/>
+    <col width="39.8" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="19.8" customWidth="1" min="6" max="6"/>
+    <col width="22.8" customWidth="1" min="6" max="6"/>
     <col width="25.1" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
     <col width="42" customWidth="1" min="11" max="11"/>
-    <col width="37.4" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -599,17 +600,17 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>OpenBMI（54 人，公开）</t>
+          <t>主办方指定标准数据集（6 人，Challenge MI）</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>被试独立五折 · test 试次级 Acc_paper（16,200 试次，每类 5,400）</t>
+          <t>LOSO6 · leave-fold 嵌套 Val（主读数）</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>E1f 四成员融合 + 因果平滑（C 臂，主结果）</t>
+          <t>E1f-A59 从零（nested-S0 / N0；**交卷终态 S0**）</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -618,25 +619,29 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.6188</v>
+        <v>0.5111</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0.6188</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>0.8094</v>
-      </c>
-      <c r="J5" s="4" t="n">
-        <v>0.6196</v>
+        <v>0.5111</v>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>判定延迟 t̄≈3.50 s；单窗前向 1.11 ms（RTX 5070）</t>
+          <t>CSV=submission_exp34_e1f_a59_sens_full_20260902_1930.csv</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>实验 30 + 混淆矩阵复算（本表 sheet 01）</t>
+          <t>实验 37/39/40 · sheet 11</t>
         </is>
       </c>
     </row>
@@ -646,17 +651,17 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>OpenBMI（54 人，公开）</t>
+          <t>主办方指定标准数据集（同上）</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>LOSO6 · 折内 Val（融合参数本折拟合；附报双标注）</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>E1f 四成员融合 + 多数票读出（W 臂，现行线上读出）</t>
+          <t>E1f-A59 折内（交卷栈同文件）</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -665,72 +670,74 @@
         </is>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.6125</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.6125</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>0.8062</v>
-      </c>
-      <c r="J6" s="6" t="n">
-        <v>0.6132</v>
+        <v>0.779</v>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>判定延迟 t̄≈4.00 s</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>实验 30 + 混淆矩阵复算（sheet 01）</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
+          <t>实验 34/35；嵌套对照 0.511（乐观≈+4.7pp）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1">
       <c r="B7" s="3" t="n">
         <v>3</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>OpenBMI（54 人，公开）</t>
+          <t>主办方指定标准数据集（同上）</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>LOSO6 · leave-fold 嵌套 Val（备选归档）</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>E1f 窗级 argmax（不作试次聚合）</t>
+          <t>E1f-B8-ft（OpenBMI→8ch FT；Exp39/40 §5 程序终态，交卷已风险否决）</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>窗级</t>
+          <t>试次级</t>
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>0.5925</v>
+        <v>0.54</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.5925</v>
+        <v>0.54</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.7962</v>
+        <v>0.77</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0.593</v>
+        <v>0.5319</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>单窗 100 ms 步进</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>混淆矩阵复算（sheet 01）</t>
+          <t>备选 CSV 归档；test Rest≈51% ∉ Val 支撑</t>
         </is>
       </c>
     </row>
@@ -740,17 +747,17 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>OpenBMI（54 人，公开）</t>
+          <t>主办方指定标准数据集（同上）</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>被试独立五折 · 试次级</t>
+          <t>LOSO6 · 折内 Val（备选附报）</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>ShallowFBCSPNet 3s 单模型（S3 底座）</t>
+          <t>E1f-B8-ft 折内</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -759,35 +766,31 @@
         </is>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.5876</v>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
+        <v>0.5733</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>0.5733</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>0.787</v>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>实验 20 登记表（0.5876±0.0296）</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
+          <t>实验 34；嵌套复核 0.540</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="38" customHeight="1">
       <c r="B9" s="3" t="n">
         <v>5</v>
       </c>
@@ -798,12 +801,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>被试独立五折 · 试次级</t>
+          <t>被试独立五折 · test 试次级 Acc_paper（16,200 试次，每类 5,400）</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Deep4Net 2s（11 模型基线最优）</t>
+          <t>E1f 四成员融合 + 因果平滑（C 臂，主结果）</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -812,25 +815,25 @@
         </is>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.5431</v>
+        <v>0.6188</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>0.5605</v>
+        <v>0.6188</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.7754</v>
+        <v>0.8094</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0.5324</v>
+        <v>0.6196</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>判定延迟 t̄≈3.50 s；单窗前向 1.11 ms（RTX 5070）</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>5090 十一模型对比（sheet 02）</t>
+          <t>实验 30 + 混淆矩阵复算（本表 sheet 01）</t>
         </is>
       </c>
     </row>
@@ -840,50 +843,44 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>BCI IV 2a（9 人，公开）</t>
+          <t>OpenBMI（54 人，公开）</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Leave-Next 6 轮仿真 · 末档（R5）· 三分类含空闲</t>
+          <t>同上</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>E1f 四成员 + all4 采后增量微调（force）</t>
+          <t>E1f 四成员融合 + 多数票读出（W 臂，现行线上读出）</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>窗级（heldout run）</t>
+          <t>试次级</t>
         </is>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.671</v>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.6125</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.6125</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>0.8062</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>0.6132</v>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>判定延迟 t̄≈4.00 s</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>实验 32（sheet 03）</t>
+          <t>实验 30 + 混淆矩阵复算（sheet 01）</t>
         </is>
       </c>
     </row>
@@ -893,17 +890,17 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>BCI IV 2a（9 人，公开）</t>
+          <t>OpenBMI（54 人，公开）</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>同上（底座零样本 R0）</t>
+          <t>同上</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>E1f 四成员零样本</t>
+          <t>E1f 窗级 argmax（不作试次聚合）</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -912,31 +909,25 @@
         </is>
       </c>
       <c r="G11" s="4" t="n">
-        <v>0.338</v>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.5925</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0.5925</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0.7962</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>0.593</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>单窗 100 ms 步进</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>实验 32（sheet 03）</t>
+          <t>混淆矩阵复算（sheet 01）</t>
         </is>
       </c>
     </row>
@@ -946,17 +937,17 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Stieger2021（24 人，公开）</t>
+          <t>OpenBMI（54 人，公开）</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>跨库伪在线 · 前半训练后半评测</t>
+          <t>被试独立五折 · 试次级</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Shallow 3s 零样本（跨库）</t>
+          <t>ShallowFBCSPNet 3s 单模型（S3 底座）</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -965,7 +956,7 @@
         </is>
       </c>
       <c r="G12" s="6" t="n">
-        <v>0.4198</v>
+        <v>0.5876</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
@@ -989,7 +980,7 @@
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>实验 07（sheet 04）</t>
+          <t>实验 20 登记表（0.5876±0.0296）</t>
         </is>
       </c>
     </row>
@@ -999,17 +990,17 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Stieger2021（24 人，公开）</t>
+          <t>OpenBMI（54 人，公开）</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>被试独立五折 · 试次级</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Shallow 3s + 前半增量微调（FT）</t>
+          <t>Deep4Net 2s（11 模型基线最优）</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -1018,60 +1009,54 @@
         </is>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.659</v>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
+        <v>0.5431</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>0.5605</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>0.7754</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>0.5324</v>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>实验 07（24/24 被试 ≥+3pp）</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
+          <t>5090 十一模型对比（sheet 02）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="38" customHeight="1">
       <c r="B14" s="5" t="n">
         <v>10</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Stieger2021（24 人，公开）</t>
+          <t>BCI IV 2a（9 人，公开）</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>同上 + 生理门控 H1</t>
+          <t>Leave-Next 6 轮仿真 · 末档（R5）· 三分类含空闲</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Shallow 3s FT + ERD 门控</t>
+          <t>E1f 四成员 + all4 采后增量微调（force）</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>试次级</t>
+          <t>窗级（heldout run）</t>
         </is>
       </c>
       <c r="G14" s="6" t="n">
-        <v>0.7003</v>
+        <v>0.663</v>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
@@ -1095,36 +1080,36 @@
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>实验 07（sheet 04）</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="38" customHeight="1">
+          <t>实验 32 stamp=20260901_124502（sheet 03）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
       <c r="B15" s="3" t="n">
         <v>11</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>自采（syj0828，8 通道 v3 范式）</t>
+          <t>BCI IV 2a（9 人，公开）</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Leave-Next 采后增量微调 · 末档（R5）</t>
+          <t>同上（底座零样本 R0）</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>E1f all4 个体模型（真实被试最优）</t>
+          <t>E1f 四成员零样本</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>窗级 heldout</t>
+          <t>窗级</t>
         </is>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.916</v>
+        <v>0.338</v>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
@@ -1143,89 +1128,308 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>MI 试次 34/36=94.4%；Rest 16/18；总分 42/45</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>复验 20260830（sheet 05）</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="38" customHeight="1">
+          <t>实验 32（sheet 03）</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
       <c r="B16" s="5" t="n">
         <v>12</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>自采（fnz0828 等其余被试）</t>
+          <t>Stieger2021（24 人，公开）</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
+          <t>跨库伪在线 · 前半训练后半评测</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Shallow 3s 零样本（跨库）</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>试次级</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>0.4198</v>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>实验 07（sheet 04）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="B17" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Stieger2021（24 人，公开）</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Shallow 3s + 前半增量微调（FT）</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>试次级</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>实验 07（24/24 被试 ≥+3pp）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="B18" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Stieger2021（24 人，公开）</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>同上 + 生理门控 H1</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Shallow 3s FT + ERD 门控</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>试次级</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>0.7003</v>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>实验 07（sheet 04）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="38" customHeight="1">
+      <c r="B19" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>自采（syj0828，8 通道 v3 范式）</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Leave-Next 采后增量微调 · 末档（R5）</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>E1f all4 个体模型（真实被试最优）</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>窗级 heldout（smooth）</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>0.924</v>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>F5 41.5/45；MI 33/36；Rest 17/18；门控 5/5 PASS</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>Leave-Next all4 全表 20260831_233943（sheet 05）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="38" customHeight="1">
+      <c r="B20" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>自采（其余 v3 被试，含 ytl0901）</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>同上 · 10 人全表</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>E1f all4 个体模型</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>窗级 heldout</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>0.35–0.69（见 sheet 05）</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>0.35–0.54（见 sheet 05）</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
-        <is>
-          <t>个体差异大，体现少样本适配必要性</t>
-        </is>
-      </c>
-      <c r="L16" s="5" t="inlineStr">
-        <is>
-          <t>复验 20260830（sheet 05）</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1"/>
-    <row r="18" ht="22" customHeight="1">
-      <c r="B18" s="7" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>门控合计 20/50 PASS；个体差异大</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>Leave-Next all4 全表</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1"/>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>注 1：OpenBMI 五折 test 划分为被试独立划分，指标为 test 试次级 Acc_paper（每试次一次判定）。</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>注 2：召回率 macro = 三类召回率均值；特异性 macro = 三类特异性均值；每类明细与混淆矩阵见 sheet 01/02。</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>注 3：主办方指定标准数据集如与本报告数据集规格不同，将以同一管线重切窗复测并回填（见 sheet 09 复现说明）。</t>
+    <row r="23" ht="22" customHeight="1">
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>注 2：召回率 macro = 三类召回率均值；特异性 macro = 三类特异性均值；每类明细与混淆矩阵见 sheet 01/02/11。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>注 3：指定集**交卷=S0**（E1f-A59 从零）：主读嵌套 0.511，折内 0.558 双标注。R-B8 nested=0.540 为 Exp39/40 备选归档（风险否决：test 预测 Rest≈51% 落在 Val 六折支撑外）。详见 sheet 07/11。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>注 4：指定集交卷栈为从零训练；OpenBMI 预训练用于系统底座/线上叙事，不作为指定集交卷依赖。赛规未禁止预训练微调，本队指定集路径选择从零以降低合规与外推风险。</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1567,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>experiment_game/data/sim_subjects/_analysis/exp32_20260829_235900/</t>
+          <t>experiment_game/data/sim_subjects/_analysis/exp32_20260901_124502/</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1407,7 +1611,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>experiment_game/data/subjects/syj0828/models/ft_runs/20260830_230014_…_summary.json</t>
+          <t>experiment_game/data/subjects/syj0828/models/ft_runs/20260831_224229_…_summary.json</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -1483,15 +1687,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="33.09999999999999" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="33.8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="9.100000000000001" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -1660,14 +1864,14 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0.671</v>
+        <v>0.663</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.671</v>
+        <v>0.663</v>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>实验 32 P1 总表</t>
+          <t>实验 32 stamp=20260901_124502 P1 总表</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -1703,32 +1907,654 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
+    <row r="12" ht="38" customHeight="1">
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>真被试 syj0828 末档窗级</t>
+          <t>真被试 syj0828 末档窗级 smooth</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>0.916</v>
+        <v>0.924</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>0.916</v>
+        <v>0.924</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>restfix 复验 20260830</t>
+          <t>leave_next_all4_full_report_20260831_233943</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
           <t>✓ PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>指定集工程主读 nested-S0（交卷）</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Exp37 N0 / Exp40 交卷</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>✓ PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>指定集备选 nested R-B8</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Exp39/40 归档</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>✓ 备选</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>指定集折内乐观（S0）</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+4.7pp</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>0.558→0.511</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Exp34 折内 vs Exp37 嵌套</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>✓ 已标注</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="19.6" customWidth="1" min="3" max="3"/>
+    <col width="16.4" customWidth="1" min="4" max="4"/>
+    <col width="14.4" customWidth="1" min="5" max="5"/>
+    <col width="18.9" customWidth="1" min="6" max="6"/>
+    <col width="34.09999999999999" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1"/>
+    <row r="2" ht="32" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>主办方指定集 · Exp34–40 诚实口径与工程终态（2026-09-04 回填）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>实验</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>臂 / 结论</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>读数</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>尺子</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>过线/采纳</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>E1f-A59（S0）</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>0.558±0.069</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>折内</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>历史主 CSV</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>科学叙事对照；嵌套后 0.511</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>E1f-B8-ft</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>0.573±0.140</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>折内</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>对照 CSV</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>嵌套复核 0.540（Exp39）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>S0 定稿</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>维持 0.558 折内</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>折内 Wilcoxon</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>科学 KEEP（后修正）</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Q1 显著性含拟合不对称；以 37/38 为准</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>M7 / M7_ABC</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>0.604 / 0.626</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>折内</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>未过 p=0.062</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>禁止作预期；嵌套后≈0.523/0.510</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>N0 nested-S0</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>0.511±0.066</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>嵌套</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>对照锚</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>折内乐观 ≈+4.7pp</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>N7 nested M7</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>0.523±0.125</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>嵌套</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>未过 p=0.81</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>弱阳性不换卷</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>G* / V1</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>0.528±0.130</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>嵌套</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>未过 p=0.69</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>仅 b8_shallow_b；选池阴性</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>R-B8</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>0.540±0.146</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>嵌套</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>工程选卷</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>非显著性；科学仍 KEEP_S0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>MC-B8</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>0.540（b≡0）</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>嵌套</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>平手→最简否决</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Rest 偏斜不可校</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>TTA-B8</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>0.538（−0.2pp）</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>嵌套</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>未进候选</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>向内缩 δ∈{0,20,40}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>终态（§5 程序）</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>R-B8_raw</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>工程规则</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>归档</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>与 Exp39 CSV 字节相同</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="38" customHeight="1">
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>**交卷（风险否决）**</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>**S0**</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Val 外推诊断</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>**采纳**</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>test Rest≈51%∉Val；无 0.300 前科</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1"/>
+    <row r="18" ht="22" customHeight="1">
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>交卷=S0（nested 0.511 + 折内 0.558 双标注）。R-B8=0.540 为备选。风险否决未改 Val 门槛、未用 test 标签调参。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1"/>
+    <row r="20" ht="24" customHeight="1">
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>R-B8 嵌套 OOF 混淆矩阵（900 试次；行=真，列=预；类序约 L/R/Rest 依 dump 标签）</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="B21" s="2" t="inlineStr"/>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>pred0</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>pred1</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>pred2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>true0</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>181</v>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>true1</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>71</v>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>196</v>
+      </c>
+      <c r="E23" s="10" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>true2</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="n">
+        <v>86</v>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>105</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1"/>
+    <row r="26" ht="22" customHeight="1">
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Acc=0.540 · recall macro=0.540 · specificity macro≈0.770 · F1 macro≈0.532（Exp39 OOF）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>风险：S0↔R-B8 test Hamming 45%；test 边际 S0 29/44/47 vs R-B8 38/21/61；若 test≈40/40/40 边际上限约 90.8%/82.5%。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:H2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2938,7 +3764,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>BCI IV 2a（A01–A09）· Leave-Next 采后增量微调仿真（实验 32）</t>
+          <t>BCI IV 2a（A01–A09）· Leave-Next 采后增量微调仿真（实验 32 · stamp=20260901_124502）</t>
         </is>
       </c>
     </row>
@@ -2984,13 +3810,13 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>0.525</v>
+        <v>0.501</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0.644</v>
+        <v>0.649</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.119</v>
+        <v>0.148</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>0.283</v>
@@ -3003,13 +3829,13 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.437</v>
+        <v>0.495</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.545</v>
+        <v>0.556</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.108</v>
+        <v>0.061</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>0.351</v>
@@ -3022,13 +3848,13 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>0.381</v>
+        <v>0.379</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>0.763</v>
+        <v>0.737</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.382</v>
+        <v>0.358</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>0.283</v>
@@ -3041,13 +3867,13 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0.423</v>
+        <v>0.47</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.636</v>
+        <v>0.642</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.213</v>
+        <v>0.172</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>0.323</v>
@@ -3060,13 +3886,13 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>0.51</v>
+        <v>0.49</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>0.621</v>
+        <v>0.578</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0.111</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>0.313</v>
@@ -3079,13 +3905,13 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.48</v>
+        <v>0.473</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.643</v>
+        <v>0.649</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.163</v>
+        <v>0.176</v>
       </c>
       <c r="F11" s="6" t="n">
         <v>0.275</v>
@@ -3098,13 +3924,13 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>0.452</v>
+        <v>0.455</v>
       </c>
       <c r="D12" s="4" t="n">
         <v>0.6889999999999999</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>0.237</v>
+        <v>0.234</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>0.379</v>
@@ -3120,10 +3946,10 @@
         <v>0.386</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>0.73</v>
+        <v>0.707</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>0.344</v>
+        <v>0.321</v>
       </c>
       <c r="F13" s="6" t="n">
         <v>0.379</v>
@@ -3136,13 +3962,13 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>0.413</v>
+        <v>0.418</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>0.764</v>
+        <v>0.756</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0.351</v>
+        <v>0.338</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>0.455</v>
@@ -3155,13 +3981,13 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>0.445</v>
+        <v>0.452</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>0.671</v>
+        <v>0.663</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>0.225</v>
+        <v>0.211</v>
       </c>
       <c r="F15" s="6" t="n">
         <v>0.338</v>
@@ -3220,13 +4046,13 @@
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>0.379</v>
+        <v>0.376</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>0.546</v>
+        <v>0.536</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>0.167</v>
+        <v>0.161</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
@@ -3236,13 +4062,13 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>0.424</v>
+        <v>0.423</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>0.607</v>
+        <v>0.593</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>0.183</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
@@ -3252,13 +4078,13 @@
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>0.395</v>
+        <v>0.392</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>0.601</v>
+        <v>0.61</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>0.207</v>
+        <v>0.218</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
@@ -3268,13 +4094,13 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>0.382</v>
+        <v>0.391</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>0.642</v>
+        <v>0.636</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0.259</v>
+        <v>0.245</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -3284,27 +4110,27 @@
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>0.445</v>
+        <v>0.452</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>0.671</v>
+        <v>0.663</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>0.225</v>
+        <v>0.211</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1"/>
     <row r="26" ht="22" customHeight="1">
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>协议：A01–A09 的 T.mat，每被试 6 轮 Leave-Next（训练=已完成 run，评测=下一 run），因果平滑 lookback=2，门控 FAIL 强制晋升（force），replay=0.10。</t>
+          <t>协议：A01–A09 的 T.mat，每被试 6 轮 Leave-Next（训练=已完成 run，评测=下一 run），因果平滑 lookback=2，门控 FAIL 强制晋升（force），replay=0.10。stamp=20260901_124502。</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>结论：all4 末档 0.671 vs so 0.445（Δ+0.225），通过预注册 +2pp 门槛 → 线上默认 FT 范围=all4（冻结 F8b）。</t>
+          <t>结论：all4 末档 0.663 vs so 0.452（Δ+0.211），通过预注册 +2pp 门槛 → 线上默认 FT 范围=all4；相对旧跑 20260829_235900 末档均值差约 ±1pp。</t>
         </is>
       </c>
     </row>
@@ -4136,34 +4962,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="8.4" customWidth="1" min="5" max="5"/>
-    <col width="10.1" customWidth="1" min="6" max="6"/>
-    <col width="10.4" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="17.7" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="10.4" customWidth="1" min="9" max="9"/>
+    <col width="18.5" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>自采真实被试 · Leave-Next 采后增量微调（F5 读出复验 2026-08-30）</t>
+          <t>自采真实被试 · Leave-Next all4（方案 A · 全表 20260831_233943 + ytl0901）</t>
         </is>
       </c>
     </row>
     <row r="3" ht="8" customHeight="1"/>
-    <row r="4" ht="24" customHeight="1">
-      <c r="B4" s="11" t="inlineStr">
-        <is>
-          <t>① 末档（各被试最后一轮 heldout 会话）结果</t>
+    <row r="4" ht="54" customHeight="1">
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>① 末档（各被试最后一轮 heldout）· FT all4 · 展示=smooth / 门控=raw · F5 试次计分</t>
         </is>
       </c>
     </row>
@@ -4180,32 +5006,32 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>窗级准确率</t>
+          <t>窗级 smooth</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>MI 试次</t>
+          <t>F5 总分</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>MI 准确率</t>
+          <t>Left</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Rest 判定</t>
+          <t>Right</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>会话总分</t>
+          <t>Rest</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>门控</t>
+          <t>门控 PASS</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -4222,19 +5048,21 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>R5（hold ws06）</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="D6" s="12" t="n">
-        <v>0.916</v>
+        <v>0.924</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>34/36</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>0.944</v>
+          <t>41.5/45</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>17/18</t>
+        </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
@@ -4243,12 +5071,12 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>42.0/45.0</t>
+          <t>17/18</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -4265,81 +5093,85 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>R4（hold ws06）</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="D7" s="13" t="n">
-        <v>0.487</v>
+        <v>0.453</v>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>15/36</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>0.417</v>
+          <t>18.0/45</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>12/18</t>
+        </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>13/18</t>
+          <t>0/18</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>21.5/45.0</t>
+          <t>12/18</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Rest 高、MI 弱</t>
+          <t>Rest 高、Right 弱</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>wzr0830</t>
+          <t>cyy0830</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>R5（hold ws06）</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="D8" s="12" t="n">
-        <v>0.541</v>
+        <v>0.409</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>12/36</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="n">
-        <v>0.333</v>
+          <t>22.5/45</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>15/18</t>
+        </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>23/36</t>
+          <t>4/18</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>23.5/54.0</t>
+          <t>7/18</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>R4 曾 0.622 PASS</t>
+          <t>含半场 w03</t>
         </is>
       </c>
     </row>
@@ -4351,76 +5183,80 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>R5（hold ws06）</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="D9" s="13" t="n">
-        <v>0.606</v>
+        <v>0.357</v>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>1/27</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>0.037</v>
+          <t>11.0/44</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>3/17</t>
+        </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>26/26</t>
+          <t>0/18</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>14.0/40.0</t>
+          <t>16/18</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>窗级升但 MI 弱</t>
+          <t>末档回落</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>xj0830</t>
+          <t>wzr0830</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>R5（hold ws06）</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="D10" s="12" t="n">
-        <v>0.522</v>
+        <v>0.425</v>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>6/35</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="n">
-        <v>0.171</v>
+          <t>17.0/45</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>26/34</t>
+          <t>3/18</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>19.0/52.0</t>
+          <t>10/18</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
@@ -4432,38 +5268,40 @@
     <row r="11" ht="22" customHeight="1">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>cyy0830</t>
+          <t>xj0830</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>R5（hold w06）</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="D11" s="13" t="n">
-        <v>0.35</v>
+        <v>0.483</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>10/36</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>0.278</v>
+          <t>20.0/45</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>14/18</t>
+        </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>7/18</t>
+          <t>1/18</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>13.5/45.0</t>
+          <t>10/18</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
@@ -4472,103 +5310,283 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1"/>
-    <row r="13" ht="24" customHeight="1">
-      <c r="B13" s="11" t="inlineStr">
+    <row r="12" ht="22" customHeight="1">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>cjf0831</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="n">
+        <v>0.468</v>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>22.0/45</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>10/18</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>8/18</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>npl0831</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="n">
+        <v>0.542</v>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>26.0/45</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>15/18</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>12/18</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>4/5</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>次优个体</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>ycx0831</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="n">
+        <v>0.418</v>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>19.0/45</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>14/18</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>3/18</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>4/18</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>2/5</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>排除半场 w06</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>ytl0901</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="n">
+        <v>0.461</v>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>23.5/45</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>12/18</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>2/5</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>w02+w03 合并为一场</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1"/>
+    <row r="17" ht="24" customHeight="1">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>② all4 vs so 消融（实验 33，末档 MI 试次准确率）</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="B14" s="2" t="inlineStr">
+    <row r="18" ht="28" customHeight="1">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>被试</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>e1f_all4_force MI</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>e1f_so_force MI</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>ΔMI</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="3" t="inlineStr">
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>syj0828</t>
         </is>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C19" s="12" t="n">
         <v>0.944</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D19" s="12" t="n">
         <v>0.222</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E19" s="12" t="n">
         <v>0.722</v>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="5" t="inlineStr">
+    <row r="20" ht="22" customHeight="1">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>fnz0828</t>
         </is>
       </c>
-      <c r="C16" s="13" t="n">
+      <c r="C20" s="13" t="n">
         <v>0.417</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D20" s="13" t="n">
         <v>0.056</v>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E20" s="13" t="n">
         <v>0.361</v>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="3" t="inlineStr">
+    <row r="21" ht="22" customHeight="1">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>两人平均</t>
         </is>
       </c>
-      <c r="C17" s="12" t="n">
+      <c r="C21" s="12" t="n">
         <v>0.681</v>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="D21" s="12" t="n">
         <v>0.139</v>
       </c>
-      <c r="E17" s="12" t="n">
+      <c r="E21" s="12" t="n">
         <v>0.542</v>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1"/>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>读出（冻结 F5）：E1f 融合概率 → 因果平滑 lookback=2 → argmax；试次 = 多数票；MI 判对 +1、专用 Rest 判对 +0.5。</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>被试爬坡示例（syj0828，窗级 heldout）：R1 0.665 → R2 0.707 → R3 0.744 → R4 0.751 → R5 0.916。</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>个体差异大（0.35–0.92）正是少样本个性化适配必要性的直接证据；门控 FAIL 时强制晋升并落盘告警（冻结 F8）。</t>
+    <row r="22" ht="22" customHeight="1"/>
+    <row r="23" ht="22" customHeight="1">
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>读出（冻结 F5 / 方案 A）：展示 heldout_acc=因果平滑；门控=raw；试次=因果平滑+多数票；MI +1、Rest +0.5。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>被试爬坡示例（syj0828，窗级 smooth）：R1 0.663 → R2 0.717 → R3 0.759 → R4 0.785 → R5 0.924。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>全表门控 20/50 PASS；个体差异大（0.35–0.92）正是少样本个性化适配必要性的直接证据；门控 FAIL 时强制晋升并落盘告警。</t>
         </is>
       </c>
     </row>
@@ -4871,7 +5889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4882,7 +5900,7 @@
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="44" customWidth="1" min="7" max="7"/>
     <col width="44" customWidth="1" min="8" max="8"/>
-    <col width="22.4" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -5062,7 +6080,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="38" customHeight="1">
+    <row r="8" ht="70" customHeight="1">
       <c r="B8" s="5" t="inlineStr">
         <is>
           <t>自采数据（OpenBCI Cyton）</t>
@@ -5075,7 +6093,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>截至 2026-08-30：9 名真实被试（6 名 v3 范式多会话 + 3 名早期范式）；【提交前更新人数】</t>
+          <t>截至 2026-09-01：≥10 名 v3 范式真实被试（syj0828/fnz0828/cyy0830/fnz0830/wzr0830/xj0830/cjf0831/npl0831/ycx0831/ytl0901 等）+ 早期范式被试；【提交前更新人数】</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -5090,7 +6108,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>采集层 0.5–45Hz 带通 + 50Hz 陷波 → LSL 推流 → CAR → 8–30Hz → 250Hz → 逐窗 z-score</t>
+          <t>采集层 0.5–45Hz 带通 + 50Hz 陷波 → LSL 推流 → CAR → 8–30Hz → 250Hz → 逐窗 z-score；EEG 看门狗 stall 2s / abort 5s</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -5104,45 +6122,45 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="38" customHeight="1">
+    <row r="9" ht="54" customHeight="1">
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>主办方指定标准数据集</t>
+          <t>主办方指定标准数据集（Challenge MI）</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>待主办方确认/发放</t>
+          <t>主办方发放；**交卷栈=59ch 从零 E1f-A59（S0）**；OpenBMI 预训练仅用于系统底座/公开库叙事（非指定集交卷依赖）</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6 被试 · LOSO6 · 每折 Val 150 试次（共 900）· 1 trial=1 窗 3s@250Hz</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>交卷 59ch 从零；备选 8 导（Pz 代 CPz，OpenBMI→FT）已归档</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>250 Hz</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>如规格与本管线不同，仅改切窗配置即可复测（管线已参数化）</t>
+          <t>与 OpenBMI 同切窗口径；轨 A：59ch 从零（交卷）；轨 B：OpenBMI→8ch FT（备选）</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>按主办方协议</t>
+          <t>被试独立 LOSO6；主读=leave-fold 嵌套 Val；折内双标注</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>【回填：60 分项主体】</t>
+          <t>60 分项主体 · 交卷 S0 nested=0.511 / 折内 0.558（Exp40 风险否决回退）</t>
         </is>
       </c>
     </row>
@@ -5151,6 +6169,13 @@
       <c r="B11" s="7" t="inlineStr">
         <is>
           <t>统一口径：通道序同时作为模型输入通道轴顺序，所有数据集、训练、微调与在线推理均不重排（通道索引 0=Cz, 1=C3, 2=C4, 3=CP3, 4=FC4, 5=FC3, 6=CP4, 7=CPz）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>交卷说明：指定集行为从零训练（S0）。OpenBMI 预训练是系统底座资产；R-B8 因 Val 支撑外推风险否决，CSV 保留归档不删。</t>
         </is>
       </c>
     </row>
@@ -5168,11 +6193,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="18.2" customWidth="1" min="2" max="2"/>
+    <col width="22.5" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
@@ -5289,7 +6314,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="38" customHeight="1">
+    <row r="10" ht="54" customHeight="1">
       <c r="B10" s="5" t="inlineStr">
         <is>
           <t>实验 32</t>
@@ -5297,12 +6322,12 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>BCI2a Leave-Next 双底座双门控仿真（all4 0.671）</t>
+          <t>BCI2a Leave-Next 双底座双门控仿真（all4 force R5=0.663 vs so 0.452）</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>资料/模型训练/32_旁路_bci2a_LeaveNext_双底座双门控_openbmi_accpaper/总结/结果登记表.md</t>
+          <t>资料/模型训练/32_旁路_bci2a_LeaveNext_双底座双门控_openbmi_accpaper/总结/结果登记表.md · 原始 exp32_20260901_124502/</t>
         </is>
       </c>
     </row>
@@ -5360,32 +6385,202 @@
     <row r="14" ht="38" customHeight="1">
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>真被试复验</t>
+          <t>真被试 Leave-Next 全表</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Leave-Next F5 restfix 逐被试明细（6 人）</t>
+          <t>10 人 all4 · 门控 20/50 · syj R5 smooth 0.924</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>experiment_game/data/subjects/_analysis/leave_next_f5_restfix_20260830_231249.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
+          <t>experiment_game/data/subjects/_analysis/leave_next_all4_full_report_20260831_233943.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="38" customHeight="1">
       <c r="B15" s="3" t="inlineStr">
         <is>
+          <t>实验 34</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>指定集 LOSO6 · E1f-A59 折内 0.558 · E1f-B8-ft 折内 0.573</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>资料/模型训练/34_旁路_挑战杯官方集_59ch离线_openbmi协议_accpaper/总结/结果登记表.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="38" customHeight="1">
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>实验 35</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>排名翻转消融 · S0 定稿（折内尺子）</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>资料/模型训练/35_旁路_官方vsOpenBMI_三分类排名不一致_融合重标定与骨干消融_accpaper/总结/结果登记表.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="38" customHeight="1">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>实验 36</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>折内跨轨融合最高 0.626（未过 Wilcoxon；后由 37 证伪为伪影）</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>资料/模型训练/36_旁路_官方主交卷_扩池与跨轨融合_accpaper/总结/结果登记表.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="38" customHeight="1">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>实验 37</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>嵌套确认 · N0=0.511 · N7=0.523 p=0.81 · 维持 S0 纪律</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>资料/模型训练/37_旁路_官方主交卷_嵌套融合McNemar确认_accpaper/总结/结果登记表.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="38" customHeight="1">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>实验 38</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>多样性选池阴性 · G*=b8_shallow_b 0.528</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>资料/模型训练/38_旁路_官方主交卷_误差去相关选池_accpaper/总结/结果登记表.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="38" customHeight="1">
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>实验 39</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>诚实排行榜 · R-B8 nested=0.540 · 工程选卷</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>资料/模型训练/39_旁路_官方主交卷_收尾回放与工程选卷_accpaper/总结/结果登记表.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="38" customHeight="1">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>实验 40</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>CSV 加固阴性 · 终态 R-B8_raw · 算法冻结</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>资料/模型训练/40_旁路_官方主交卷_CSV加固_边际校正与TTA_accpaper/总结/结果登记表.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="38" customHeight="1">
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>指定集工程 CSV</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>submission_exp40_rb8_raw_final_*（=Exp39 R-B8）</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>code/train_lab/out/5070_challenge_exp40_csv_harden_tta_accpaper/submissions/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>指定集回退 CSV</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Exp34 S0</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>code/train_lab/out/5070_challenge_mi_59ch_accpaper/submissions/submission_exp34_e1f_a59_sens_full_20260902_1930.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>统计口径方案 A</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>展示=smooth · 门控=raw · F5 试次计分</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>experiment_game/docs/统计口径方案A_20260831.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="B25" s="3" t="inlineStr">
+        <is>
           <t>框架冻结</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>现行系统口径（F1–F25）</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>experiment_game/docs/框架冻结确认_20260829.md</t>
         </is>

</xml_diff>

<commit_message>
docs: adopt QuadFold-59 / CausalFuse-8 as public model names
Sync prelim report, Excel, video script, and Exp34–41 registries to the frozen outward names while keeping internal S0/E1f paths unchanged.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/资料/初赛材料/02_离线验证/离线性能验证报告_XH-202610.xlsx
+++ b/资料/初赛材料/02_离线验证/离线性能验证报告_XH-202610.xlsx
@@ -610,7 +610,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>E1f-A59 从零（nested-S0 / N0；**交卷终态 S0**）</t>
+          <t>QuadFold-59（nested / 内部 S0·E1f-A59；**交卷终态**）</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>E1f-A59 折内（交卷栈同文件）</t>
+          <t>QuadFold-59 折内（交卷栈同文件）</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>E1f 四成员融合 + 因果平滑（C 臂，主结果）</t>
+          <t>CausalFuse-8 + 因果滑窗（C 臂，主结果）</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>E1f 四成员融合 + 多数票读出（W 臂，现行线上读出）</t>
+          <t>CausalFuse-8 + 多数票读出（W 臂，现行线上读出）</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>E1f 窗级 argmax（不作试次聚合）</t>
+          <t>CausalFuse-8 窗级 argmax（不作试次聚合）</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>E1f 四成员 + all4 采后增量微调（force）</t>
+          <t>CausalFuse-8FT（all4 采后增量微调 force）</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>E1f 四成员零样本</t>
+          <t>CausalFuse-8 零样本</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>E1f all4 个体模型（真实被试最优）</t>
+          <t>CausalFuse-8FT 个体模型（真实被试最优）</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>E1f all4 个体模型</t>
+          <t>CausalFuse-8FT 个体模型</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -1422,14 +1422,14 @@
     <row r="24" ht="22" customHeight="1">
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>注 3：指定集**交卷=S0**（E1f-A59 从零）：主读嵌套 0.511，折内 0.558 双标注。R-B8 nested=0.540 为 Exp39/40 备选归档（风险否决：test 预测 Rest≈51% 落在 Val 六折支撑外）。详见 sheet 07/11。</t>
+          <t>注 3：指定集**交卷=QuadFold-59**（内部 S0 / E1f-A59）：主读嵌套 0.511，折内 0.558 双标注。R-B8 nested=0.540 为 Exp39/40 备选归档（风险否决：test 预测 Rest≈51% 落在 Val 六折支撑外）。详见 sheet 07/11。</t>
         </is>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>注 4：指定集交卷栈为从零训练；OpenBMI 预训练用于系统底座/线上叙事，不作为指定集交卷依赖。赛规未禁止预训练微调，本队指定集路径选择从零以降低合规与外推风险。</t>
+          <t>注 4：QuadFold-59 为从零训练交卷；CausalFuse-8 为 OpenBMI 预训练在线底座，不作为指定集交卷依赖。赛规未禁止预训练微调，本队指定集路径选择从零以降低合规与外推风险。</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>主结果复现：E1f 各臂混淆矩阵与每类指标（自动对账锚点 0.6125/0.6188）</t>
+          <t>主结果复现：CausalFuse-8 各臂混淆矩阵与每类指标（自动对账锚点 0.6125/0.6188）</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1691,7 +1691,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="33.09999999999999" customWidth="1" min="2" max="2"/>
+    <col width="39.70000000000001" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
@@ -1780,7 +1780,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="38" customHeight="1">
+    <row r="7" ht="22" customHeight="1">
       <c r="B7" s="3" t="inlineStr">
         <is>
           <t>macro 召回 = 总体准确率（类别均衡）</t>
@@ -1930,10 +1930,10 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1">
+    <row r="13" ht="38" customHeight="1">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>指定集工程主读 nested-S0（交卷）</t>
+          <t>指定集工程主读 QuadFold-59 nested（交卷）</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
@@ -2023,7 +2023,7 @@
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
     <col width="19.6" customWidth="1" min="3" max="3"/>
-    <col width="16.4" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="14.4" customWidth="1" min="5" max="5"/>
     <col width="18.9" customWidth="1" min="6" max="6"/>
     <col width="34.09999999999999" customWidth="1" min="7" max="7"/>
@@ -2079,7 +2079,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>E1f-A59（S0）</t>
+          <t>QuadFold-59（S0）</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>**S0**</t>
+          <t>**QuadFold-59**</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -2459,7 +2459,7 @@
     <row r="18" ht="22" customHeight="1">
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>交卷=S0（nested 0.511 + 折内 0.558 双标注）。R-B8=0.540 为备选。风险否决未改 Val 门槛、未用 test 标签调参。</t>
+          <t>交卷=QuadFold-59（nested 0.511 + 折内 0.558 双标注）。R-B8=0.540 为备选。风险否决未改 Val 门槛、未用 test 标签调参。</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2585,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>OpenBMI 54 人五折 · E1f 主结果明细（混淆矩阵与每类指标）</t>
+          <t>OpenBMI 54 人五折 · CausalFuse-8 主结果明细（混淆矩阵与每类指标）</t>
         </is>
       </c>
     </row>
@@ -2593,7 +2593,7 @@
     <row r="4" ht="38" customHeight="1">
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>① 主结果：E1f 四成员 + 因果平滑（C 臂）试次判定 · test 集准确率 0.6188（对账锚点一致）</t>
+          <t>① 主结果：CausalFuse-8 + 因果滑窗（C 臂）试次判定 · test 集准确率 0.6188（对账锚点一致）</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
     <row r="31" ht="22" customHeight="1">
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>E1f 四成员融合 · 窗级 argmax</t>
+          <t>CausalFuse-8 · 窗级 argmax</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
@@ -3728,7 +3728,7 @@
     <row r="19" ht="22" customHeight="1">
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>3s 主线补充：Shallow 3s 单模型三分类 0.5876±0.0296（Task 二分类 0.7415±0.0306）；E1f 四成员融合三分类 0.6173（classic 臂）→ 因果平滑 0.6188（C 臂，见 sheet 01）。</t>
+          <t>3s 主线补充：Shallow 3s 单模型三分类 0.5876±0.0296（Task 二分类 0.7415±0.0306）；CausalFuse-8 融合三分类 0.6173（classic 臂）→ 因果滑窗 0.6188（C 臂，见 sheet 01）。</t>
         </is>
       </c>
     </row>
@@ -6130,7 +6130,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>主办方发放；**交卷栈=59ch 从零 E1f-A59（S0）**；OpenBMI 预训练仅用于系统底座/公开库叙事（非指定集交卷依赖）</t>
+          <t>主办方发放；**交卷栈=QuadFold-59**（内部 S0/E1f-A59）；CausalFuse-8 仅用于系统底座/公开库叙事（非指定集交卷依赖）</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>与 OpenBMI 同切窗口径；轨 A：59ch 从零（交卷）；轨 B：OpenBMI→8ch FT（备选）</t>
+          <t>与 OpenBMI 同切窗口径；轨 A：QuadFold-59（交卷）；轨 B：OpenBMI→8ch FT（备选）</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>60 分项主体 · 交卷 S0 nested=0.511 / 折内 0.558（Exp40 风险否决回退）</t>
+          <t>60 分项主体 · 交卷 QuadFold-59 nested=0.511 / 折内 0.558（Exp40 风险否决回退）</t>
         </is>
       </c>
     </row>
@@ -6175,7 +6175,7 @@
     <row r="12" ht="22" customHeight="1">
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>交卷说明：指定集行为从零训练（S0）。OpenBMI 预训练是系统底座资产；R-B8 因 Val 支撑外推风险否决，CSV 保留归档不删。</t>
+          <t>交卷说明：指定集交卷=QuadFold-59（从零）。CausalFuse-8 是系统底座资产；R-B8 因 Val 支撑外推风险否决，CSV 保留归档不删。</t>
         </is>
       </c>
     </row>
@@ -6237,7 +6237,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>E1f 各臂 W/classic/S/C replay（0.6125/0.6173/0.6170/0.6188）</t>
+          <t>CausalFuse-8 各臂 W/classic/S/C replay（0.6125/0.6173/0.6170/0.6188）</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -6305,7 +6305,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>E1f 四成员融合 0.6173（classic）与配置</t>
+          <t>CausalFuse-8（E1f）四成员融合 0.6173（classic）与配置</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -6407,7 +6407,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>指定集 LOSO6 · E1f-A59 折内 0.558 · E1f-B8-ft 折内 0.573</t>
+          <t>指定集 LOSO6 · QuadFold-59 折内 0.558 · E1f-B8-ft 折内 0.573</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">

</xml_diff>